<commit_message>
Estado metas y contribución corte 202608
</commit_message>
<xml_diff>
--- a/main_data/contrafactual_num_clientes_con_uso.xlsx
+++ b/main_data/contrafactual_num_clientes_con_uso.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -466,348 +466,854 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>45292</v>
+        <v>44562</v>
       </c>
       <c r="B2" t="n">
-        <v>2540.983660146594</v>
+        <v>99829.29393115958</v>
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="n">
-        <v>2221</v>
+        <v>100138</v>
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>45323</v>
+        <v>44593</v>
       </c>
       <c r="B3" t="n">
-        <v>5691.441176488996</v>
+        <v>108610.876364474</v>
       </c>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="n">
-        <v>5779</v>
+        <v>109024</v>
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>45352</v>
+        <v>44621</v>
       </c>
       <c r="B4" t="n">
-        <v>8841.898692816496</v>
+        <v>115298.6261015855</v>
       </c>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="n">
-        <v>9282</v>
+        <v>116036</v>
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>45383</v>
+        <v>44652</v>
       </c>
       <c r="B5" t="n">
-        <v>11992.3562091589</v>
+        <v>120911.5312706205</v>
       </c>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="n">
-        <v>12131</v>
+        <v>121448</v>
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>45413</v>
+        <v>44682</v>
       </c>
       <c r="B6" t="n">
-        <v>15142.8137255013</v>
+        <v>126012.9869675448</v>
       </c>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="n">
-        <v>15160</v>
+        <v>126439</v>
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>45444</v>
+        <v>44713</v>
       </c>
       <c r="B7" t="n">
-        <v>18293.2712418437</v>
+        <v>130653.1745231934</v>
       </c>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="n">
-        <v>17724</v>
+        <v>130903</v>
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>45474</v>
+        <v>44743</v>
       </c>
       <c r="B8" t="n">
-        <v>21443.7287581712</v>
+        <v>135319.9041553524</v>
       </c>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="n">
-        <v>20987</v>
+        <v>135132</v>
       </c>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>45505</v>
+        <v>44774</v>
       </c>
       <c r="B9" t="n">
-        <v>24594.1862745136</v>
+        <v>140056.0228979619</v>
       </c>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="n">
-        <v>24050</v>
+        <v>139704</v>
       </c>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>45536</v>
+        <v>44805</v>
       </c>
       <c r="B10" t="n">
-        <v>27744.643790856</v>
+        <v>144972.404639437</v>
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="n">
-        <v>27744</v>
+        <v>144479</v>
       </c>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>45566</v>
+        <v>44835</v>
       </c>
       <c r="B11" t="n">
-        <v>30895.10130719841</v>
+        <v>149547.0050710909</v>
       </c>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="n">
-        <v>31092</v>
+        <v>148966</v>
       </c>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>45597</v>
+        <v>44866</v>
       </c>
       <c r="B12" t="n">
-        <v>34045.55882354081</v>
+        <v>154284.1938677915</v>
       </c>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="n">
-        <v>34340</v>
+        <v>153457</v>
       </c>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>45627</v>
+        <v>44896</v>
       </c>
       <c r="B13" t="n">
-        <v>37196.01633986831</v>
+        <v>158810.9688376944</v>
       </c>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="n">
-        <v>37912</v>
+        <v>157445</v>
       </c>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>45658</v>
+        <v>44927</v>
       </c>
       <c r="B14" t="n">
-        <v>268.2849673330784</v>
+        <v>107793.0829483807</v>
       </c>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="n">
-        <v>1532</v>
+        <v>107477</v>
       </c>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>45689</v>
+        <v>44958</v>
       </c>
       <c r="B15" t="n">
-        <v>3418.74248367548</v>
+        <v>116558.3181352473</v>
       </c>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="n">
-        <v>3760</v>
+        <v>115938</v>
       </c>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>45717</v>
+        <v>44986</v>
       </c>
       <c r="B16" t="n">
-        <v>6569.200000017881</v>
+        <v>122979.0537324779</v>
       </c>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="n">
-        <v>6196</v>
+        <v>122262</v>
       </c>
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>45748</v>
+        <v>45017</v>
       </c>
       <c r="B17" t="n">
-        <v>9719.657516345382</v>
+        <v>128177.4999344965</v>
       </c>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="n">
-        <v>9031</v>
+        <v>126957</v>
       </c>
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>45778</v>
+        <v>45047</v>
       </c>
       <c r="B18" t="n">
-        <v>12870.11503268778</v>
+        <v>132768.9258991437</v>
       </c>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="n">
-        <v>12327</v>
+        <v>131712</v>
       </c>
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>45809</v>
-      </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="n">
-        <v>16020.57254903018</v>
-      </c>
+        <v>45078</v>
+      </c>
+      <c r="B19" t="n">
+        <v>136816.4012183867</v>
+      </c>
+      <c r="C19" t="inlineStr"/>
       <c r="D19" t="n">
-        <v>15268</v>
-      </c>
-      <c r="E19" t="n">
-        <v>-752.5725490301847</v>
-      </c>
-      <c r="F19" t="n">
-        <v>-0.04697538410234547</v>
-      </c>
+        <v>136339</v>
+      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>45839</v>
-      </c>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" t="n">
-        <v>19171.03006537259</v>
-      </c>
+        <v>45108</v>
+      </c>
+      <c r="B20" t="n">
+        <v>140837.0560427765</v>
+      </c>
+      <c r="C20" t="inlineStr"/>
       <c r="D20" t="n">
-        <v>18936</v>
-      </c>
-      <c r="E20" t="n">
-        <v>-235.0300653725863</v>
-      </c>
-      <c r="F20" t="n">
-        <v>-0.01225964721619764</v>
-      </c>
+        <v>140889</v>
+      </c>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>45870</v>
-      </c>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" t="n">
-        <v>22321.48758171499</v>
-      </c>
+        <v>45139</v>
+      </c>
+      <c r="B21" t="n">
+        <v>144875.2195265789</v>
+      </c>
+      <c r="C21" t="inlineStr"/>
       <c r="D21" t="n">
-        <v>22995</v>
-      </c>
-      <c r="E21" t="n">
-        <v>673.5124182850122</v>
-      </c>
-      <c r="F21" t="n">
-        <v>0.03017327657125912</v>
-      </c>
+        <v>145321</v>
+      </c>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>45901</v>
-      </c>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" t="n">
-        <v>25471.94509804249</v>
-      </c>
+        <v>45170</v>
+      </c>
+      <c r="B22" t="n">
+        <v>149044.0764836493</v>
+      </c>
+      <c r="C22" t="inlineStr"/>
       <c r="D22" t="n">
-        <v>27900</v>
-      </c>
-      <c r="E22" t="n">
-        <v>2428.054901957512</v>
-      </c>
-      <c r="F22" t="n">
-        <v>0.09532271260054291</v>
-      </c>
+        <v>149493</v>
+      </c>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>45931</v>
-      </c>
-      <c r="B23" t="inlineStr"/>
-      <c r="C23" t="n">
-        <v>28622.40261438489</v>
-      </c>
+        <v>45200</v>
+      </c>
+      <c r="B23" t="n">
+        <v>152807.3197769355</v>
+      </c>
+      <c r="C23" t="inlineStr"/>
       <c r="D23" t="n">
-        <v>32665</v>
-      </c>
-      <c r="E23" t="n">
-        <v>4042.59738561511</v>
-      </c>
-      <c r="F23" t="n">
-        <v>0.1412389253298884</v>
-      </c>
+        <v>153331</v>
+      </c>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
+        <v>45231</v>
+      </c>
+      <c r="B24" t="n">
+        <v>156684.1025890263</v>
+      </c>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="n">
+        <v>157546</v>
+      </c>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>45261</v>
+      </c>
+      <c r="B25" t="n">
+        <v>160295.3981478311</v>
+      </c>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="n">
+        <v>161505</v>
+      </c>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>45292</v>
+      </c>
+      <c r="B26" t="n">
+        <v>108135.5548706839</v>
+      </c>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="n">
+        <v>108323</v>
+      </c>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>45323</v>
+      </c>
+      <c r="B27" t="n">
+        <v>116213.8670188846</v>
+      </c>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="n">
+        <v>117135</v>
+      </c>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>45352</v>
+      </c>
+      <c r="B28" t="n">
+        <v>121866.0929848367</v>
+      </c>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="n">
+        <v>122783</v>
+      </c>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>45383</v>
+      </c>
+      <c r="B29" t="n">
+        <v>126241.0499573871</v>
+      </c>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="n">
+        <v>126883</v>
+      </c>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>45413</v>
+      </c>
+      <c r="B30" t="n">
+        <v>129963.7708482856</v>
+      </c>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="n">
+        <v>130559</v>
+      </c>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>45444</v>
+      </c>
+      <c r="B31" t="n">
+        <v>133107.0581704311</v>
+      </c>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="n">
+        <v>133317</v>
+      </c>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>45474</v>
+      </c>
+      <c r="B32" t="n">
+        <v>136181.1261479271</v>
+      </c>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="n">
+        <v>136320</v>
+      </c>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>45505</v>
+      </c>
+      <c r="B33" t="n">
+        <v>139229.4637714896</v>
+      </c>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="n">
+        <v>139151</v>
+      </c>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>45536</v>
+      </c>
+      <c r="B34" t="n">
+        <v>142360.2769903859</v>
+      </c>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="n">
+        <v>142416</v>
+      </c>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n">
+        <v>45566</v>
+      </c>
+      <c r="B35" t="n">
+        <v>145062.5551088015</v>
+      </c>
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="n">
+        <v>145129</v>
+      </c>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>45597</v>
+      </c>
+      <c r="B36" t="n">
+        <v>147833.6022662161</v>
+      </c>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="n">
+        <v>147813</v>
+      </c>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>45627</v>
+      </c>
+      <c r="B37" t="n">
+        <v>150316.3909890218</v>
+      </c>
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="n">
+        <v>150475</v>
+      </c>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n">
+        <v>45658</v>
+      </c>
+      <c r="B38" t="n">
+        <v>100783.8301436455</v>
+      </c>
+      <c r="C38" t="inlineStr"/>
+      <c r="D38" t="n">
+        <v>100593</v>
+      </c>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n">
+        <v>45689</v>
+      </c>
+      <c r="B39" t="n">
+        <v>107650.8241681749</v>
+      </c>
+      <c r="C39" t="inlineStr"/>
+      <c r="D39" t="n">
+        <v>106961</v>
+      </c>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n">
+        <v>45717</v>
+      </c>
+      <c r="B40" t="n">
+        <v>112196.5118187556</v>
+      </c>
+      <c r="C40" t="inlineStr"/>
+      <c r="D40" t="n">
+        <v>111289</v>
+      </c>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n">
+        <v>45748</v>
+      </c>
+      <c r="B41" t="inlineStr"/>
+      <c r="C41" t="n">
+        <v>115513.8677260307</v>
+      </c>
+      <c r="D41" t="n">
+        <v>114972</v>
+      </c>
+      <c r="E41" t="n">
+        <v>-541.8677260306722</v>
+      </c>
+      <c r="F41" t="n">
+        <v>-0.004713040792807572</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n">
+        <v>45778</v>
+      </c>
+      <c r="B42" t="inlineStr"/>
+      <c r="C42" t="n">
+        <v>118193.3090673013</v>
+      </c>
+      <c r="D42" t="n">
+        <v>118446</v>
+      </c>
+      <c r="E42" t="n">
+        <v>252.6909326986643</v>
+      </c>
+      <c r="F42" t="n">
+        <v>0.002133385109658952</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n">
+        <v>45809</v>
+      </c>
+      <c r="B43" t="inlineStr"/>
+      <c r="C43" t="n">
+        <v>120311.9410876219</v>
+      </c>
+      <c r="D43" t="n">
+        <v>121329</v>
+      </c>
+      <c r="E43" t="n">
+        <v>1017.058912378066</v>
+      </c>
+      <c r="F43" t="n">
+        <v>0.008382653053911815</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n">
+        <v>45839</v>
+      </c>
+      <c r="B44" t="inlineStr"/>
+      <c r="C44" t="n">
+        <v>122338.0715554493</v>
+      </c>
+      <c r="D44" t="n">
+        <v>124484</v>
+      </c>
+      <c r="E44" t="n">
+        <v>2145.928444550664</v>
+      </c>
+      <c r="F44" t="n">
+        <v>0.01723858844952495</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="n">
+        <v>45870</v>
+      </c>
+      <c r="B45" t="inlineStr"/>
+      <c r="C45" t="n">
+        <v>124311.9617611162</v>
+      </c>
+      <c r="D45" t="n">
+        <v>127041</v>
+      </c>
+      <c r="E45" t="n">
+        <v>2729.038238883833</v>
+      </c>
+      <c r="F45" t="n">
+        <v>0.02148155507972885</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n">
+        <v>45901</v>
+      </c>
+      <c r="B46" t="inlineStr"/>
+      <c r="C46" t="n">
+        <v>126330.3369333246</v>
+      </c>
+      <c r="D46" t="n">
+        <v>129736</v>
+      </c>
+      <c r="E46" t="n">
+        <v>3405.66306667545</v>
+      </c>
+      <c r="F46" t="n">
+        <v>0.02625071735428447</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n">
+        <v>45931</v>
+      </c>
+      <c r="B47" t="inlineStr"/>
+      <c r="C47" t="n">
+        <v>127941.4337962276</v>
+      </c>
+      <c r="D47" t="n">
+        <v>132463</v>
+      </c>
+      <c r="E47" t="n">
+        <v>4521.566203772411</v>
+      </c>
+      <c r="F47" t="n">
+        <v>0.03413455986783034</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n">
         <v>45962</v>
       </c>
-      <c r="B24" t="inlineStr"/>
-      <c r="C24" t="n">
-        <v>31772.86013072729</v>
-      </c>
-      <c r="D24" t="n">
-        <v>37253</v>
-      </c>
-      <c r="E24" t="n">
-        <v>5480.139869272709</v>
-      </c>
-      <c r="F24" t="n">
-        <v>0.1724786451935722</v>
+      <c r="B48" t="inlineStr"/>
+      <c r="C48" t="n">
+        <v>129588.3948874215</v>
+      </c>
+      <c r="D48" t="n">
+        <v>134816</v>
+      </c>
+      <c r="E48" t="n">
+        <v>5227.605112578516</v>
+      </c>
+      <c r="F48" t="n">
+        <v>0.03877585088252519</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n">
+        <v>45992</v>
+      </c>
+      <c r="B49" t="inlineStr"/>
+      <c r="C49" t="n">
+        <v>130959.302007952</v>
+      </c>
+      <c r="D49" t="n">
+        <v>137535</v>
+      </c>
+      <c r="E49" t="n">
+        <v>6575.697992048023</v>
+      </c>
+      <c r="F49" t="n">
+        <v>0.047811088028851</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>46023</v>
+      </c>
+      <c r="B50" t="inlineStr"/>
+      <c r="C50" t="n">
+        <v>87268.58439242601</v>
+      </c>
+      <c r="D50" t="n">
+        <v>99964</v>
+      </c>
+      <c r="E50" t="n">
+        <v>12695.41560757399</v>
+      </c>
+      <c r="F50" t="n">
+        <v>0.1269998760311111</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>46054</v>
+      </c>
+      <c r="B51" t="inlineStr"/>
+      <c r="C51" t="n">
+        <v>92644.89464237767</v>
+      </c>
+      <c r="D51" t="n">
+        <v>106088</v>
+      </c>
+      <c r="E51" t="n">
+        <v>13443.10535762233</v>
+      </c>
+      <c r="F51" t="n">
+        <v>0.1267165500115219</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>46082</v>
+      </c>
+      <c r="B52" t="inlineStr"/>
+      <c r="C52" t="n">
+        <v>95966.69715168916</v>
+      </c>
+      <c r="D52" t="n">
+        <v>110281</v>
+      </c>
+      <c r="E52" t="n">
+        <v>14314.30284831084</v>
+      </c>
+      <c r="F52" t="n">
+        <v>0.1297984498536542</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B53" t="inlineStr"/>
+      <c r="C53" t="n">
+        <v>98200.20155406055</v>
+      </c>
+      <c r="D53" t="n">
+        <v>113583</v>
+      </c>
+      <c r="E53" t="n">
+        <v>15382.79844593945</v>
+      </c>
+      <c r="F53" t="n">
+        <v>0.1354322252972668</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B54" t="inlineStr"/>
+      <c r="C54" t="n">
+        <v>99863.82719280467</v>
+      </c>
+      <c r="D54" t="n">
+        <v>116521</v>
+      </c>
+      <c r="E54" t="n">
+        <v>16657.17280719533</v>
+      </c>
+      <c r="F54" t="n">
+        <v>0.1429542555178494</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B55" t="inlineStr"/>
+      <c r="C55" t="n">
+        <v>101032.5020575746</v>
+      </c>
+      <c r="D55" t="n">
+        <v>119036</v>
+      </c>
+      <c r="E55" t="n">
+        <v>18003.49794242543</v>
+      </c>
+      <c r="F55" t="n">
+        <v>0.1512441441448421</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B56" t="inlineStr"/>
+      <c r="C56" t="n">
+        <v>102105.9535649014</v>
+      </c>
+      <c r="D56" t="n">
+        <v>121439</v>
+      </c>
+      <c r="E56" t="n">
+        <v>19333.04643509864</v>
+      </c>
+      <c r="F56" t="n">
+        <v>0.1591996511425378</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B57" t="inlineStr"/>
+      <c r="C57" t="n">
+        <v>103119.1716783954</v>
+      </c>
+      <c r="D57" t="n">
+        <v>123775</v>
+      </c>
+      <c r="E57" t="n">
+        <v>20655.82832160455</v>
+      </c>
+      <c r="F57" t="n">
+        <v>0.1668820708673363</v>
       </c>
     </row>
   </sheetData>

</xml_diff>